<commit_message>
Update Excel test case reports and security audit findings
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.047</v>
+        <v>0.097</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.074</v>
+        <v>0.121</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.089</v>
+        <v>0.1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.054</v>
+        <v>0.119</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.117</v>
+        <v>0.095</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.077</v>
+        <v>0.132</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.045</v>
+        <v>0.101</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.116</v>
+        <v>0.062</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.05</v>
+        <v>0.143</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.1</v>
+        <v>0.123</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.149</v>
+        <v>0.135</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.12</v>
+        <v>0.153</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.043</v>
+        <v>0.061</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.135</v>
+        <v>0.037</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.047</v>
+        <v>0.141</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.081</v>
+        <v>0.115</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.148</v>
+        <v>0.115</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.053</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.14</v>
+        <v>0.136</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.132</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.124</v>
+        <v>0.08</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.055</v>
+        <v>0.034</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.038</v>
+        <v>0.107</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.118</v>
+        <v>0.111</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.105</v>
+        <v>0.028</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.104</v>
+        <v>0.115</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.062</v>
+        <v>0.091</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.06</v>
+        <v>0.042</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.118</v>
+        <v>0.078</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.028</v>
+        <v>0.117</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.06</v>
+        <v>0.083</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.107</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0.03</v>
+        <v>0.034</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>0.053</v>
+        <v>0.076</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0.057</v>
+        <v>0.077</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.079</v>
+        <v>0.073</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0.012</v>
+        <v>0.045</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.036</v>
+        <v>0.015</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0.019</v>
+        <v>0.05</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0.019</v>
+        <v>0.037</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.064</v>
+        <v>0.079</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0.05</v>
+        <v>0.034</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.043</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>0.078</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>0.017</v>
+        <v>0.077</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.076</v>
+        <v>0.06</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.079</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>0.256</v>
+        <v>0.167</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0.132</v>
+        <v>0.305</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2254,7 +2254,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.205</v>
+        <v>0.231</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.161</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.132</v>
+        <v>0.281</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0.244</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>0.122</v>
+        <v>0.288</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0.107</v>
+        <v>0.097</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>0.125</v>
+        <v>0.11</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>0.134</v>
+        <v>0.245</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0.211</v>
+        <v>0.236</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>

</xml_diff>